<commit_message>
chore(weekly-sync): auto-pull through 2026-06-11
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week23.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week23.xlsx
@@ -731,7 +731,7 @@
         <v>43</v>
       </c>
       <c r="F11" t="n">
-        <v>13395</v>
+        <v>13394</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -1095,7 +1095,7 @@
         <v>27</v>
       </c>
       <c r="F24" t="n">
-        <v>1853</v>
+        <v>1852</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -1129,7 +1129,7 @@
         <v>26811.92</v>
       </c>
       <c r="H25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26">
@@ -1266,10 +1266,10 @@
         <v>25140</v>
       </c>
       <c r="G30" t="n">
-        <v>60978.91</v>
+        <v>63223.83</v>
       </c>
       <c r="H30" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31">
@@ -1431,7 +1431,7 @@
         <v>51</v>
       </c>
       <c r="F36" t="n">
-        <v>8519</v>
+        <v>8517</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -1490,10 +1490,10 @@
         <v>7323</v>
       </c>
       <c r="G38" t="n">
-        <v>6250</v>
+        <v>7689.83</v>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
@@ -1767,7 +1767,7 @@
         <v>254</v>
       </c>
       <c r="F48" t="n">
-        <v>46608</v>
+        <v>46606</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -1829,7 +1829,7 @@
         <v>12200.84</v>
       </c>
       <c r="H50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
@@ -1845,13 +1845,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2859.41</v>
+        <v>2856.57</v>
       </c>
       <c r="E51" t="n">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F51" t="n">
-        <v>47487</v>
+        <v>47485</v>
       </c>
       <c r="G51" t="n">
         <v>28555.92</v>
@@ -1938,10 +1938,10 @@
         <v>81814</v>
       </c>
       <c r="G54" t="n">
-        <v>55200</v>
+        <v>59266.95</v>
       </c>
       <c r="H54" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55">
@@ -2162,10 +2162,10 @@
         <v>30851</v>
       </c>
       <c r="G62" t="n">
-        <v>32142.36</v>
+        <v>38411.86</v>
       </c>
       <c r="H62" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="63">
@@ -2190,10 +2190,10 @@
         <v>5788</v>
       </c>
       <c r="G63" t="n">
-        <v>12793.22</v>
+        <v>16012.71</v>
       </c>
       <c r="H63" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64">
@@ -2218,10 +2218,10 @@
         <v>38518</v>
       </c>
       <c r="G64" t="n">
-        <v>16603.42</v>
+        <v>19483.93</v>
       </c>
       <c r="H64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65">
@@ -2271,7 +2271,7 @@
         <v>40</v>
       </c>
       <c r="F66" t="n">
-        <v>4825</v>
+        <v>4823</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -2327,13 +2327,13 @@
         <v>137</v>
       </c>
       <c r="F68" t="n">
-        <v>15727</v>
+        <v>15726</v>
       </c>
       <c r="G68" t="n">
-        <v>6396.62</v>
+        <v>10802.55</v>
       </c>
       <c r="H68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69">
@@ -2498,10 +2498,10 @@
         <v>5208</v>
       </c>
       <c r="G74" t="n">
-        <v>4405.93</v>
+        <v>8811.860000000001</v>
       </c>
       <c r="H74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75">
@@ -2579,7 +2579,7 @@
         <v>464</v>
       </c>
       <c r="F77" t="n">
-        <v>66369</v>
+        <v>66367</v>
       </c>
       <c r="G77" t="n">
         <v>7878.81</v>
@@ -2837,7 +2837,7 @@
         <v>5676.27</v>
       </c>
       <c r="H86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
@@ -3055,7 +3055,7 @@
         <v>435</v>
       </c>
       <c r="F94" t="n">
-        <v>91084</v>
+        <v>91083</v>
       </c>
       <c r="G94" t="n">
         <v>24564.47</v>
@@ -3142,10 +3142,10 @@
         <v>47099</v>
       </c>
       <c r="G97" t="n">
-        <v>13209.3</v>
+        <v>14225.4</v>
       </c>
       <c r="H97" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="98">
@@ -3223,7 +3223,7 @@
         <v>866</v>
       </c>
       <c r="F100" t="n">
-        <v>79301</v>
+        <v>79298</v>
       </c>
       <c r="G100" t="n">
         <v>15886.44</v>
@@ -3254,10 +3254,10 @@
         <v>13685</v>
       </c>
       <c r="G101" t="n">
-        <v>46923.69</v>
+        <v>44594.03</v>
       </c>
       <c r="H101" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="102">
@@ -3441,13 +3441,13 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1279.2</v>
+        <v>1278.03</v>
       </c>
       <c r="E108" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F108" t="n">
-        <v>27997</v>
+        <v>27995</v>
       </c>
       <c r="G108" t="n">
         <v>4236.44</v>
@@ -3497,13 +3497,13 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1413.46</v>
+        <v>1409.81</v>
       </c>
       <c r="E110" t="n">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F110" t="n">
-        <v>36755</v>
+        <v>36753</v>
       </c>
       <c r="G110" t="n">
         <v>4660.17</v>
@@ -3951,7 +3951,7 @@
         <v>16</v>
       </c>
       <c r="F126" t="n">
-        <v>2157</v>
+        <v>2156</v>
       </c>
       <c r="G126" t="n">
         <v>0</v>
@@ -4623,7 +4623,7 @@
         <v>124</v>
       </c>
       <c r="F150" t="n">
-        <v>75718</v>
+        <v>75715</v>
       </c>
       <c r="G150" t="n">
         <v>6877.98</v>
@@ -4651,7 +4651,7 @@
         <v>37</v>
       </c>
       <c r="F151" t="n">
-        <v>8481</v>
+        <v>8480</v>
       </c>
       <c r="G151" t="n">
         <v>0</v>
@@ -4679,7 +4679,7 @@
         <v>14</v>
       </c>
       <c r="F152" t="n">
-        <v>10254</v>
+        <v>10251</v>
       </c>
       <c r="G152" t="n">
         <v>0</v>
@@ -4735,7 +4735,7 @@
         <v>21</v>
       </c>
       <c r="F154" t="n">
-        <v>2771</v>
+        <v>2770</v>
       </c>
       <c r="G154" t="n">
         <v>0</v>
@@ -4819,7 +4819,7 @@
         <v>40</v>
       </c>
       <c r="F157" t="n">
-        <v>8115</v>
+        <v>8114</v>
       </c>
       <c r="G157" t="n">
         <v>0</v>
@@ -4903,7 +4903,7 @@
         <v>6</v>
       </c>
       <c r="F160" t="n">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="G160" t="n">
         <v>1694.07</v>
@@ -4987,7 +4987,7 @@
         <v>1503</v>
       </c>
       <c r="F163" t="n">
-        <v>127172</v>
+        <v>127170</v>
       </c>
       <c r="G163" t="n">
         <v>24400.87</v>
@@ -5015,7 +5015,7 @@
         <v>39</v>
       </c>
       <c r="F164" t="n">
-        <v>44482</v>
+        <v>44480</v>
       </c>
       <c r="G164" t="n">
         <v>0</v>
@@ -5071,7 +5071,7 @@
         <v>17</v>
       </c>
       <c r="F166" t="n">
-        <v>17740</v>
+        <v>17739</v>
       </c>
       <c r="G166" t="n">
         <v>0</v>
@@ -5127,7 +5127,7 @@
         <v>44</v>
       </c>
       <c r="F168" t="n">
-        <v>3521</v>
+        <v>3520</v>
       </c>
       <c r="G168" t="n">
         <v>1143.22</v>
@@ -5183,7 +5183,7 @@
         <v>1163</v>
       </c>
       <c r="F170" t="n">
-        <v>206458</v>
+        <v>206452</v>
       </c>
       <c r="G170" t="n">
         <v>35247.46</v>
@@ -5267,7 +5267,7 @@
         <v>28</v>
       </c>
       <c r="F173" t="n">
-        <v>4612</v>
+        <v>4611</v>
       </c>
       <c r="G173" t="n">
         <v>0</v>
@@ -5323,7 +5323,7 @@
         <v>12</v>
       </c>
       <c r="F175" t="n">
-        <v>2145</v>
+        <v>2144</v>
       </c>
       <c r="G175" t="n">
         <v>0</v>
@@ -5379,7 +5379,7 @@
         <v>203</v>
       </c>
       <c r="F177" t="n">
-        <v>46982</v>
+        <v>46981</v>
       </c>
       <c r="G177" t="n">
         <v>12942.37</v>
@@ -5407,7 +5407,7 @@
         <v>30</v>
       </c>
       <c r="F178" t="n">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="G178" t="n">
         <v>0</v>
@@ -5463,7 +5463,7 @@
         <v>16</v>
       </c>
       <c r="F180" t="n">
-        <v>7492</v>
+        <v>7489</v>
       </c>
       <c r="G180" t="n">
         <v>2117.8</v>
@@ -5491,7 +5491,7 @@
         <v>7</v>
       </c>
       <c r="F181" t="n">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="G181" t="n">
         <v>0</v>
@@ -5631,7 +5631,7 @@
         <v>289</v>
       </c>
       <c r="F186" t="n">
-        <v>60254</v>
+        <v>60249</v>
       </c>
       <c r="G186" t="n">
         <v>1312.71</v>
@@ -5653,13 +5653,13 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>502.18</v>
+        <v>501.18</v>
       </c>
       <c r="E187" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F187" t="n">
-        <v>30607</v>
+        <v>30605</v>
       </c>
       <c r="G187" t="n">
         <v>2498.3</v>
@@ -5883,7 +5883,7 @@
         <v>31</v>
       </c>
       <c r="F195" t="n">
-        <v>6034</v>
+        <v>6033</v>
       </c>
       <c r="G195" t="n">
         <v>0</v>
@@ -5961,13 +5961,13 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>185.46</v>
+        <v>182.06</v>
       </c>
       <c r="E198" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F198" t="n">
-        <v>10136</v>
+        <v>10134</v>
       </c>
       <c r="G198" t="n">
         <v>4744.06</v>
@@ -6163,7 +6163,7 @@
         <v>109</v>
       </c>
       <c r="F205" t="n">
-        <v>27396</v>
+        <v>27395</v>
       </c>
       <c r="G205" t="n">
         <v>2509.34</v>
@@ -6247,13 +6247,13 @@
         <v>344</v>
       </c>
       <c r="F208" t="n">
-        <v>71041</v>
+        <v>71040</v>
       </c>
       <c r="G208" t="n">
-        <v>2032.2</v>
+        <v>3048.3</v>
       </c>
       <c r="H208" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="209">
@@ -6275,13 +6275,13 @@
         <v>193</v>
       </c>
       <c r="F209" t="n">
-        <v>62755</v>
+        <v>62754</v>
       </c>
       <c r="G209" t="n">
         <v>3388.14</v>
       </c>
       <c r="H209" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="210">
@@ -6415,7 +6415,7 @@
         <v>64</v>
       </c>
       <c r="F214" t="n">
-        <v>13849</v>
+        <v>13847</v>
       </c>
       <c r="G214" t="n">
         <v>0</v>
@@ -6471,7 +6471,7 @@
         <v>23</v>
       </c>
       <c r="F216" t="n">
-        <v>6506</v>
+        <v>6505</v>
       </c>
       <c r="G216" t="n">
         <v>0</v>
@@ -6527,7 +6527,7 @@
         <v>40</v>
       </c>
       <c r="F218" t="n">
-        <v>9050</v>
+        <v>9049</v>
       </c>
       <c r="G218" t="n">
         <v>0</v>
@@ -6891,7 +6891,7 @@
         <v>295</v>
       </c>
       <c r="F231" t="n">
-        <v>29529</v>
+        <v>29524</v>
       </c>
       <c r="G231" t="n">
         <v>21014.41</v>
@@ -6919,7 +6919,7 @@
         <v>197</v>
       </c>
       <c r="F232" t="n">
-        <v>17276</v>
+        <v>17275</v>
       </c>
       <c r="G232" t="n">
         <v>0</v>
@@ -6947,7 +6947,7 @@
         <v>71</v>
       </c>
       <c r="F233" t="n">
-        <v>14855</v>
+        <v>14853</v>
       </c>
       <c r="G233" t="n">
         <v>0</v>
@@ -7171,7 +7171,7 @@
         <v>2330</v>
       </c>
       <c r="F241" t="n">
-        <v>303391</v>
+        <v>303385</v>
       </c>
       <c r="G241" t="n">
         <v>17240.67</v>
@@ -7227,7 +7227,7 @@
         <v>471</v>
       </c>
       <c r="F243" t="n">
-        <v>39871</v>
+        <v>39870</v>
       </c>
       <c r="G243" t="n">
         <v>11015.26</v>
@@ -7249,19 +7249,19 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>2233.25</v>
+        <v>2232.25</v>
       </c>
       <c r="E244" t="n">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="F244" t="n">
-        <v>122371</v>
+        <v>122368</v>
       </c>
       <c r="G244" t="n">
-        <v>13034.74</v>
+        <v>16423.72</v>
       </c>
       <c r="H244" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="245">
@@ -7333,13 +7333,13 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>732.98</v>
+        <v>731.98</v>
       </c>
       <c r="E247" t="n">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F247" t="n">
-        <v>32080</v>
+        <v>32078</v>
       </c>
       <c r="G247" t="n">
         <v>4236.44</v>
@@ -7367,7 +7367,7 @@
         <v>77</v>
       </c>
       <c r="F248" t="n">
-        <v>12954</v>
+        <v>12953</v>
       </c>
       <c r="G248" t="n">
         <v>3388.98</v>
@@ -7395,7 +7395,7 @@
         <v>342</v>
       </c>
       <c r="F249" t="n">
-        <v>39979</v>
+        <v>39976</v>
       </c>
       <c r="G249" t="n">
         <v>4660.17</v>
@@ -7445,19 +7445,19 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>10353.93</v>
+        <v>10352.93</v>
       </c>
       <c r="E251" t="n">
-        <v>3900</v>
+        <v>3899</v>
       </c>
       <c r="F251" t="n">
-        <v>399752</v>
+        <v>399747</v>
       </c>
       <c r="G251" t="n">
-        <v>21861.03</v>
+        <v>22411.03</v>
       </c>
       <c r="H251" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="252">
@@ -7678,10 +7678,10 @@
         <v>32226</v>
       </c>
       <c r="G259" t="n">
-        <v>23725.44</v>
+        <v>30080.52</v>
       </c>
       <c r="H259" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="260">
@@ -7762,10 +7762,10 @@
         <v>23235</v>
       </c>
       <c r="G262" t="n">
-        <v>17662.7</v>
+        <v>19992.36</v>
       </c>
       <c r="H262" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="263">
@@ -7983,7 +7983,7 @@
         <v>32</v>
       </c>
       <c r="F270" t="n">
-        <v>4882</v>
+        <v>4881</v>
       </c>
       <c r="G270" t="n">
         <v>0</v>
@@ -8039,13 +8039,13 @@
         <v>114</v>
       </c>
       <c r="F272" t="n">
-        <v>33716</v>
+        <v>33714</v>
       </c>
       <c r="G272" t="n">
-        <v>3388.98</v>
+        <v>6777.96</v>
       </c>
       <c r="H272" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="273">
@@ -8089,13 +8089,13 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>1306.34</v>
+        <v>1291.28</v>
       </c>
       <c r="E274" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F274" t="n">
-        <v>16461</v>
+        <v>16459</v>
       </c>
       <c r="G274" t="n">
         <v>0</v>
@@ -8210,10 +8210,10 @@
         <v>48389</v>
       </c>
       <c r="G278" t="n">
-        <v>46381.44</v>
+        <v>48626.36</v>
       </c>
       <c r="H278" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="279">
@@ -8465,7 +8465,7 @@
         <v>6776.28</v>
       </c>
       <c r="H287" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="288">
@@ -8633,7 +8633,7 @@
         <v>4516.67</v>
       </c>
       <c r="H293" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="294">
@@ -8689,7 +8689,7 @@
         <v>5123.74</v>
       </c>
       <c r="H295" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="296">
@@ -9103,7 +9103,7 @@
         <v>95</v>
       </c>
       <c r="F310" t="n">
-        <v>36591</v>
+        <v>36589</v>
       </c>
       <c r="G310" t="n">
         <v>3219.49</v>
@@ -9187,7 +9187,7 @@
         <v>47</v>
       </c>
       <c r="F313" t="n">
-        <v>8239</v>
+        <v>8238</v>
       </c>
       <c r="G313" t="n">
         <v>3033.06</v>
@@ -9246,10 +9246,10 @@
         <v>45782</v>
       </c>
       <c r="G315" t="n">
-        <v>18930.45</v>
+        <v>20299.09</v>
       </c>
       <c r="H315" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="316">
@@ -9349,19 +9349,19 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>9345.82</v>
+        <v>9343.33</v>
       </c>
       <c r="E319" t="n">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="F319" t="n">
-        <v>134463</v>
+        <v>134457</v>
       </c>
       <c r="G319" t="n">
-        <v>32064.47</v>
+        <v>34309.39</v>
       </c>
       <c r="H319" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="320">
@@ -9439,7 +9439,7 @@
         <v>447</v>
       </c>
       <c r="F322" t="n">
-        <v>155594</v>
+        <v>155593</v>
       </c>
       <c r="G322" t="n">
         <v>5122.88</v>
@@ -9523,7 +9523,7 @@
         <v>26</v>
       </c>
       <c r="F325" t="n">
-        <v>6427</v>
+        <v>6426</v>
       </c>
       <c r="G325" t="n">
         <v>0</v>
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>201.41</v>
+        <v>193.41</v>
       </c>
       <c r="E326" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F326" t="n">
-        <v>4853</v>
+        <v>4851</v>
       </c>
       <c r="G326" t="n">
         <v>4489.83</v>
@@ -9719,7 +9719,7 @@
         <v>68</v>
       </c>
       <c r="F332" t="n">
-        <v>8104</v>
+        <v>8103</v>
       </c>
       <c r="G332" t="n">
         <v>13598.29</v>
@@ -10111,7 +10111,7 @@
         <v>61</v>
       </c>
       <c r="F346" t="n">
-        <v>8200</v>
+        <v>8198</v>
       </c>
       <c r="G346" t="n">
         <v>0</v>
@@ -10251,7 +10251,7 @@
         <v>693</v>
       </c>
       <c r="F351" t="n">
-        <v>65929</v>
+        <v>65928</v>
       </c>
       <c r="G351" t="n">
         <v>21120.8</v>
@@ -10335,7 +10335,7 @@
         <v>9</v>
       </c>
       <c r="F354" t="n">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="G354" t="n">
         <v>0</v>
@@ -10615,7 +10615,7 @@
         <v>20</v>
       </c>
       <c r="F364" t="n">
-        <v>1829</v>
+        <v>1828</v>
       </c>
       <c r="G364" t="n">
         <v>677.12</v>
@@ -11259,7 +11259,7 @@
         <v>6</v>
       </c>
       <c r="F387" t="n">
-        <v>1509</v>
+        <v>1507</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
@@ -11287,7 +11287,7 @@
         <v>12</v>
       </c>
       <c r="F388" t="n">
-        <v>1791</v>
+        <v>1790</v>
       </c>
       <c r="G388" t="n">
         <v>0</v>
@@ -11623,7 +11623,7 @@
         <v>19</v>
       </c>
       <c r="F400" t="n">
-        <v>3175</v>
+        <v>3174</v>
       </c>
       <c r="G400" t="n">
         <v>0</v>
@@ -12015,7 +12015,7 @@
         <v>33</v>
       </c>
       <c r="F414" t="n">
-        <v>6253</v>
+        <v>6252</v>
       </c>
       <c r="G414" t="n">
         <v>0</v>
@@ -12071,7 +12071,7 @@
         <v>124</v>
       </c>
       <c r="F416" t="n">
-        <v>11724</v>
+        <v>11723</v>
       </c>
       <c r="G416" t="n">
         <v>17455.93</v>
@@ -12494,10 +12494,10 @@
         <v>17537</v>
       </c>
       <c r="G431" t="n">
-        <v>21522.88</v>
+        <v>1355.08</v>
       </c>
       <c r="H431" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="432">
@@ -12774,10 +12774,10 @@
         <v>30984</v>
       </c>
       <c r="G441" t="n">
-        <v>7454.23</v>
+        <v>9316.939999999999</v>
       </c>
       <c r="H441" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="442">
@@ -12802,10 +12802,10 @@
         <v>50828</v>
       </c>
       <c r="G442" t="n">
-        <v>25844.09</v>
+        <v>31816.98</v>
       </c>
       <c r="H442" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="443">
@@ -12849,13 +12849,13 @@
         </is>
       </c>
       <c r="D444" t="n">
-        <v>773.88</v>
+        <v>765.88</v>
       </c>
       <c r="E444" t="n">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F444" t="n">
-        <v>10911</v>
+        <v>10910</v>
       </c>
       <c r="G444" t="n">
         <v>12173.34</v>
@@ -12942,10 +12942,10 @@
         <v>25906</v>
       </c>
       <c r="G447" t="n">
-        <v>0</v>
+        <v>11438.98</v>
       </c>
       <c r="H447" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="448">
@@ -13275,7 +13275,7 @@
         <v>12</v>
       </c>
       <c r="F459" t="n">
-        <v>2172</v>
+        <v>2171</v>
       </c>
       <c r="G459" t="n">
         <v>0</v>
@@ -13415,7 +13415,7 @@
         <v>2</v>
       </c>
       <c r="F464" t="n">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="G464" t="n">
         <v>0</v>
@@ -13443,7 +13443,7 @@
         <v>19</v>
       </c>
       <c r="F465" t="n">
-        <v>2924</v>
+        <v>2923</v>
       </c>
       <c r="G465" t="n">
         <v>0</v>
@@ -13471,7 +13471,7 @@
         <v>103</v>
       </c>
       <c r="F466" t="n">
-        <v>20919</v>
+        <v>20918</v>
       </c>
       <c r="G466" t="n">
         <v>0</v>
@@ -13527,7 +13527,7 @@
         <v>21</v>
       </c>
       <c r="F468" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="G468" t="n">
         <v>0</v>
@@ -13555,7 +13555,7 @@
         <v>11</v>
       </c>
       <c r="F469" t="n">
-        <v>2165</v>
+        <v>2164</v>
       </c>
       <c r="G469" t="n">
         <v>0</v>
@@ -13617,7 +13617,7 @@
         <v>11711.71</v>
       </c>
       <c r="H471" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="472">
@@ -13695,13 +13695,13 @@
         <v>136</v>
       </c>
       <c r="F474" t="n">
-        <v>23527</v>
+        <v>23526</v>
       </c>
       <c r="G474" t="n">
-        <v>5501.7</v>
+        <v>6051.7</v>
       </c>
       <c r="H474" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="475">
@@ -13863,7 +13863,7 @@
         <v>184</v>
       </c>
       <c r="F480" t="n">
-        <v>39997</v>
+        <v>39994</v>
       </c>
       <c r="G480" t="n">
         <v>15161.97</v>
@@ -13891,7 +13891,7 @@
         <v>44</v>
       </c>
       <c r="F481" t="n">
-        <v>12864</v>
+        <v>12863</v>
       </c>
       <c r="G481" t="n">
         <v>0</v>
@@ -13975,7 +13975,7 @@
         <v>133</v>
       </c>
       <c r="F484" t="n">
-        <v>36715</v>
+        <v>36710</v>
       </c>
       <c r="G484" t="n">
         <v>8748.309999999999</v>
@@ -14031,13 +14031,13 @@
         <v>43</v>
       </c>
       <c r="F486" t="n">
-        <v>10689</v>
+        <v>10688</v>
       </c>
       <c r="G486" t="n">
-        <v>1694.07</v>
+        <v>3405.09</v>
       </c>
       <c r="H486" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="487">
@@ -14115,7 +14115,7 @@
         <v>15</v>
       </c>
       <c r="F489" t="n">
-        <v>4620</v>
+        <v>4619</v>
       </c>
       <c r="G489" t="n">
         <v>2456.78</v>
@@ -14227,7 +14227,7 @@
         <v>58</v>
       </c>
       <c r="F493" t="n">
-        <v>14348</v>
+        <v>14347</v>
       </c>
       <c r="G493" t="n">
         <v>0</v>
@@ -14255,7 +14255,7 @@
         <v>35</v>
       </c>
       <c r="F494" t="n">
-        <v>7424</v>
+        <v>7423</v>
       </c>
       <c r="G494" t="n">
         <v>1694.07</v>
@@ -14283,7 +14283,7 @@
         <v>59</v>
       </c>
       <c r="F495" t="n">
-        <v>9285</v>
+        <v>9284</v>
       </c>
       <c r="G495" t="n">
         <v>1694.07</v>
@@ -14339,7 +14339,7 @@
         <v>13</v>
       </c>
       <c r="F497" t="n">
-        <v>4756</v>
+        <v>4755</v>
       </c>
       <c r="G497" t="n">
         <v>0</v>
@@ -14395,7 +14395,7 @@
         <v>28</v>
       </c>
       <c r="F499" t="n">
-        <v>7586</v>
+        <v>7585</v>
       </c>
       <c r="G499" t="n">
         <v>0</v>
@@ -14423,7 +14423,7 @@
         <v>156</v>
       </c>
       <c r="F500" t="n">
-        <v>34080</v>
+        <v>34079</v>
       </c>
       <c r="G500" t="n">
         <v>10333.91</v>
@@ -14451,13 +14451,13 @@
         <v>45</v>
       </c>
       <c r="F501" t="n">
-        <v>14830</v>
+        <v>14829</v>
       </c>
       <c r="G501" t="n">
-        <v>1778.81</v>
+        <v>3854.23</v>
       </c>
       <c r="H501" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="502">
@@ -14669,13 +14669,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4303.29</v>
+        <v>4294.85</v>
       </c>
       <c r="E6" t="n">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F6" t="n">
-        <v>80380</v>
+        <v>80374</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -14697,19 +14697,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2030.41</v>
+        <v>2027.15</v>
       </c>
       <c r="E7" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F7" t="n">
         <v>69081</v>
       </c>
       <c r="G7" t="n">
-        <v>13552.54</v>
+        <v>16940.68</v>
       </c>
       <c r="H7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -14731,7 +14731,7 @@
         <v>698</v>
       </c>
       <c r="F8" t="n">
-        <v>195962</v>
+        <v>195960</v>
       </c>
       <c r="G8" t="n">
         <v>5802.55</v>
@@ -14899,13 +14899,13 @@
         <v>640</v>
       </c>
       <c r="F14" t="n">
-        <v>170599</v>
+        <v>170594</v>
       </c>
       <c r="G14" t="n">
-        <v>39705.09</v>
+        <v>41399.16</v>
       </c>
       <c r="H14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -14955,7 +14955,7 @@
         <v>215</v>
       </c>
       <c r="F16" t="n">
-        <v>79023</v>
+        <v>79021</v>
       </c>
       <c r="G16" t="n">
         <v>10843.24</v>
@@ -15005,10 +15005,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>821.6</v>
+        <v>820.5699999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F18" t="n">
         <v>49510</v>
@@ -15291,7 +15291,7 @@
         <v>1991</v>
       </c>
       <c r="F28" t="n">
-        <v>565025</v>
+        <v>565018</v>
       </c>
       <c r="G28" t="n">
         <v>21183.9</v>
@@ -15481,13 +15481,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>3686.17</v>
+        <v>3685.16</v>
       </c>
       <c r="E35" t="n">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F35" t="n">
-        <v>152549</v>
+        <v>152543</v>
       </c>
       <c r="G35" t="n">
         <v>13654.69</v>
@@ -15543,13 +15543,13 @@
         <v>148</v>
       </c>
       <c r="F37" t="n">
-        <v>26810</v>
+        <v>26804</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>7033.05</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -15621,19 +15621,19 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>6950.3</v>
+        <v>6946.16</v>
       </c>
       <c r="E40" t="n">
-        <v>4059</v>
+        <v>4055</v>
       </c>
       <c r="F40" t="n">
-        <v>1004717</v>
+        <v>1004701</v>
       </c>
       <c r="G40" t="n">
-        <v>20250.85</v>
+        <v>34316.95</v>
       </c>
       <c r="H40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
@@ -15767,7 +15767,7 @@
         <v>504</v>
       </c>
       <c r="F45" t="n">
-        <v>148849</v>
+        <v>148841</v>
       </c>
       <c r="G45" t="n">
         <v>27574.63</v>
@@ -16175,7 +16175,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>38236</v>
+        <v>38235</v>
       </c>
       <c r="E11" t="n">
         <v>394</v>
@@ -16184,7 +16184,7 @@
         <v>6988.744211349059</v>
       </c>
       <c r="G11" t="n">
-        <v>8979.68</v>
+        <v>10679.37142362812</v>
       </c>
       <c r="H11" t="n">
         <v>5</v>
@@ -16217,10 +16217,10 @@
         <v>2241.855788650941</v>
       </c>
       <c r="G12" t="n">
-        <v>2880.51</v>
+        <v>3425.738576371879</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -16280,7 +16280,7 @@
         <v>89</v>
       </c>
       <c r="F14" t="n">
-        <v>713.6148785311477</v>
+        <v>711.8881959737676</v>
       </c>
       <c r="G14" t="n">
         <v>6777.96</v>
@@ -16313,7 +16313,7 @@
         <v>104</v>
       </c>
       <c r="F15" t="n">
-        <v>838.3518736577879</v>
+        <v>836.3233739715545</v>
       </c>
       <c r="G15" t="n">
         <v>7962.719999999999</v>
@@ -16349,7 +16349,7 @@
         <v>1315.01219351602</v>
       </c>
       <c r="G16" t="n">
-        <v>1105.94</v>
+        <v>2069.735454001105</v>
       </c>
       <c r="H16" t="n">
         <v>1</v>
@@ -16415,10 +16415,10 @@
         <v>3828.11780648398</v>
       </c>
       <c r="G18" t="n">
-        <v>3219.49</v>
+        <v>6025.184545998894</v>
       </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -16442,10 +16442,10 @@
         <v>20809</v>
       </c>
       <c r="E19" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F19" t="n">
-        <v>927.7532478110641</v>
+        <v>925.5084300546778</v>
       </c>
       <c r="G19" t="n">
         <v>8811.860000000001</v>

</xml_diff>